<commit_message>
feat: enhance chatbot prompt with cross-tab routing and welcome notice
- Add tab selection rules to system prompt so keyword-based questions route to the correct dataset regardless of active tab
- Add blue-colored notice under example questions advising users to select the relevant tab for better accuracy
- Update Q&A reference xlsx
</commit_message>
<xml_diff>
--- a/질의응답.xlsx
+++ b/질의응답.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="25">
   <si>
     <t>당월 보험수익 금액 알려줘</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -50,16 +50,40 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>951억</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>10월 보험수익 금액 알려줘</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t>943억</t>
+    <t>보험서비스비용의  전월차 얼마?</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>답변</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>정답여부</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(무)확정사망 상품의 NP 모델 당월 데이터 알려줘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>당월(202512) 보험수익은 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF48535B"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>951억</t>
     </r>
     <r>
       <rPr>
@@ -70,74 +94,138 @@
         <charset val="129"/>
         <scheme val="minor"/>
       </rPr>
-      <t> </t>
-    </r>
-  </si>
-  <si>
-    <t>19억</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>보험서비스비용의  전월차 얼마?</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>당월(202512) 보험서비스비용이 전월(202511) 대비 597억 증가했습니다.</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>| 마감년월 | 보험수익 (억) | 원본 |
-|---------|------------|------|
-| 2025년 01월 | 859억 | 859.4292 |
-| 2025년 02월 | 876억 | 875.5606 |
-| 2025년 03월 | 857억 | 857.2889 |
-| 2025년 04월 | 863억 | 862.7945 |
-| 2025년 05월 | 875억 | 875.0862 |
-| 2025년 06월 | 879억 | 879.0408 |
-| 2025년 07월 | 916억 | 915.6002 |
-| 2025년 08월 | 925억 | 924.7516 |
-| 2025년 09월 | 910억 | 910.0237 |
-| 2025년 10월 | 943억 | 943.0121 |
-| 2025년 11월 | 951억 | 950.8693 |
-| 2025년 12월 | 951억 | 950.6583 |
-| 연간 합계 | 10,905억 | 10,904.1154 |</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">01월 │ +159 │                              ┃███████████
-02월 │ +131 │                              ┃█████████
-03월 │ +135 │                              ┃█████████
-04월 │  +80 │                              ┃█████
-05월 │ +227 │                              ┃███████████████
-06월 │ +150 │                              ┃██████████
-07월 │ +145 │                              ┃██████████
-08월 │ +176 │                              ┃████████████
-09월 │  +18 │                              ┃█
-10월 │ +248 │                              ┃█████████████████
-11월 │ +160 │                              ┃███████████
-12월 │ -451 │██████████████████████████████┃
-      </t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>그래프로 보여줘</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>답변</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>정답여부</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>(무)확정사망 상품의 NP 모델 당월 데이터 알려줘</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>• 이자부리(보험금융비용): 62억
-• 부담이자율: 2.93%</t>
+      <t>입니다</t>
+    </r>
+  </si>
+  <si>
+    <t>2025년 10월 보험수익은 943억입니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>202512 NP 모델 RA변동은 보험수익 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF48535B"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>19억</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF48535B"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, 보험서비스비용 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF48535B"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>0억</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF48535B"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>입니다.</t>
+    </r>
+  </si>
+  <si>
+    <t>25.12 보험서비스비용은 1,329억, 전월('25.11) 732억 대비 +597억 증가했습니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025년 보험수익 월별 현황입니다.
+• 1월: 859억 / 2월: 876억 / 3월: 857억
+• 4월: 863억 / 5월: 875억 / 6월: 879억
+• 7월: 916억 / 8월: 925억 / 9월: 910억
+• 10월: 943억 / 11월: 951억 / 12월: 951억
+연간 합계 10,804억, 하반기로 갈수록 상승 추세를 보입니다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>현재 활성 탭(보험금융손익) 기준, 선택월 202510 (무)확정사망 NP 데이터입니다.
+• 보험금융비용(이자부리): 61억
+• 부담이자율: 2.94%</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>지급보험금 예실차 (유)확정건강의 당월 예상금액이 얼마나</t>
+  </si>
+  <si>
+    <r>
+      <t>2025년 10월 (유)확정건강의 지급보험금 예상금액은 </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF48535B"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>2억</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF48535B"/>
+        <rFont val="맑은 고딕"/>
+        <family val="3"/>
+        <charset val="129"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> (1.72억, 반올림)입니다</t>
+    </r>
+  </si>
+  <si>
+    <t>지급보험금 예실차 (유)확정건강의 당월 실금액이 얼마나</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(유)확정건강의 당월(2025.10) 지급보험금 실제 금액은 1억입니다.
+(예상 2억, Variance +1억)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>사업비 예실차 변액연금의 당월 예상금액이 얼마나</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025년 10월 기준 변액연금 사업비 예실차 예상금액은 총 67억입니다.
+• 유지비 9억, 신계약비(PL) 10억, 신계약비(CSM) 48억</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>사업비 예실차 변액연금의 당월 실금액이 얼마니</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -239,7 +327,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -261,14 +349,20 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -550,7 +644,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
@@ -567,10 +661,10 @@
         <v>5</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
@@ -580,20 +674,22 @@
       <c r="B2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>8</v>
+      <c r="C3" s="11" t="s">
+        <v>12</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>1</v>
@@ -601,13 +697,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>9</v>
+      <c r="C4" s="10" t="s">
+        <v>13</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>1</v>
@@ -618,78 +714,102 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>14</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="202.5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="108" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="8" t="s">
-        <v>12</v>
+      <c r="C6" s="7" t="s">
+        <v>15</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="264" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="82.5" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>13</v>
+        <v>10</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>16</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="33" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="10" t="s">
         <v>18</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="2"/>
+    <row r="9" spans="1:4" ht="33" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="33" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3"/>
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="C11" s="3"/>
-      <c r="D11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
-      <c r="B12" s="3"/>
+      <c r="B12" s="4" t="s">
+        <v>22</v>
+      </c>
       <c r="C12" s="3"/>
       <c r="D12" s="2"/>
     </row>
@@ -788,12 +908,6 @@
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="2"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="2"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>